<commit_message>
Se arreglo modulos como: credenciales, audiovisuales, panel operativo, multas y se dejo funcional el dashboard
</commit_message>
<xml_diff>
--- a/tmp/aulas-prueba/aulas_formato_actual.xlsx
+++ b/tmp/aulas-prueba/aulas_formato_actual.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aulas" sheetId="1" r:id="R440db715e9f74888"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aulas" sheetId="1" r:id="R7b4a5e0d366f4de4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -377,29 +377,6 @@
         <x:v>No</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="6" t="str">
-        <x:v>AULA-NUEVA-914</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:v>Diseño Industrial</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="n">
-        <x:v>2021</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="str">
-        <x:v>Dell Precision 3660</x:v>
-      </x:c>
-      <x:c r="F5" s="6" t="str">
-        <x:v>Sala para modelado y diseño</x:v>
-      </x:c>
-      <x:c r="G5" s="6" t="str">
-        <x:v>Sí</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>